<commit_message>
Milestone: SysML relations and signal connections demo on snapshot 5eaf843e
Capture shared relation/status views, historical snapshot routing, IPOS operational and reporting fixes, tests, approved working authority state, generated model/document evidence, and local handoff notes.

Verified scope: 315 affected/focused tests passed earlier; user Stage 6 and traceability/hierarchy refreshes completed with exit 0; eight selected-snapshot digital document checks passed. Snapshot: snap-73c872b1307b6adb5eaf843e. This milestone save does not rerun generation or certify final SysML implementation readiness. Current readiness evidence remains NOT_READY/NOT_ASSESSED as recorded.

Known unapplied follow-ups: Tk ThemeChanged test teardown cleanup and automatic DOCX/XLSX reopening on GUI refresh. Personal settings, source drafts, experimental proof directories, caches, lock files and local backup ZIPs are excluded.
</commit_message>
<xml_diff>
--- a/artifacts/traceability_reports/analog_ipos_vs_ars.xlsx
+++ b/artifacts/traceability_reports/analog_ipos_vs_ars.xlsx
@@ -9,10 +9,14 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analog IPOS vs ARS" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report Metadata" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upstream Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Presence" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analog IPOS vs ARS'!$A$1:$A$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Analog IPOS vs ARS'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Upstream Coverage'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Requirement Presence'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0&quot;%&quot;"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -63,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -73,6 +79,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -147,6 +154,51 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReportData2" displayName="ReportData2" ref="A1:P2" headerRowCount="1">
+  <autoFilter ref="A1:P2"/>
+  <tableColumns count="16">
+    <tableColumn id="1" name="covering_level"/>
+    <tableColumn id="2" name="covering_block"/>
+    <tableColumn id="3" name="covered_upstream_level"/>
+    <tableColumn id="4" name="covered_upstream_block"/>
+    <tableColumn id="5" name="denominator_scope"/>
+    <tableColumn id="6" name="covered_unique_upstream_requirements"/>
+    <tableColumn id="7" name="total_unique_upstream_requirements"/>
+    <tableColumn id="8" name="uncovered_upstream_requirements"/>
+    <tableColumn id="9" name="coverage_percentage"/>
+    <tableColumn id="10" name="coverage_status"/>
+    <tableColumn id="11" name="coverage_basis"/>
+    <tableColumn id="12" name="covered_upstream_requirement_ids"/>
+    <tableColumn id="13" name="uncovered_upstream_requirement_ids"/>
+    <tableColumn id="14" name="snapshot_id"/>
+    <tableColumn id="15" name="covering_node_id"/>
+    <tableColumn id="16" name="covered_upstream_node_id"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ReportData3" displayName="ReportData3" ref="A1:K2" headerRowCount="1">
+  <autoFilter ref="A1:K2"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="hierarchy_level"/>
+    <tableColumn id="2" name="block"/>
+    <tableColumn id="3" name="scope"/>
+    <tableColumn id="4" name="expected_requirements"/>
+    <tableColumn id="5" name="represented_requirements"/>
+    <tableColumn id="6" name="missing_requirements"/>
+    <tableColumn id="7" name="presence_percentage"/>
+    <tableColumn id="8" name="presence_status"/>
+    <tableColumn id="9" name="coverage_basis"/>
+    <tableColumn id="10" name="missing_requirement_ids"/>
+    <tableColumn id="11" name="snapshot_id"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -499,7 +551,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09T15:20:02+00:00</t>
+          <t>2026-10-15T20:02:17+00:00</t>
         </is>
       </c>
     </row>
@@ -588,4 +640,325 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="31" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>covering_level</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>covering_block</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>covered_upstream_level</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>covered_upstream_block</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>denominator_scope</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>covered_unique_upstream_requirements</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>total_unique_upstream_requirements</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>uncovered_upstream_requirements</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>coverage_percentage</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>coverage_status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>coverage_basis</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>covered_upstream_requirement_ids</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>uncovered_upstream_requirement_ids</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>snapshot_id</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>covering_node_id</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>covered_upstream_node_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Analog IPOS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>(All blocks)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>(All blocks)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No approved upstream relationship</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>no_applicable_relationship</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>No approved upstream relationship in central graph; no coverage denominator inferred</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>snap-73c872b1307b6adb5eaf843e</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Analog IPOS</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="31" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>hierarchy_level</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>block</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>expected_requirements</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>represented_requirements</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>missing_requirements</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>presence_percentage</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>presence_status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>coverage_basis</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>missing_requirement_ids</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>snapshot_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Analog IPOS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>(All blocks)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Level total</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>valid_empty</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Approved allocation IDs represented in target traceability matrix</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>snap-73c872b1307b6adb5eaf843e</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>